<commit_message>
Cash flow forecast: proposed template structure, project sections, flow-type bug fix
</commit_message>
<xml_diff>
--- a/public/cash-flow-forecast-unze-trading.xlsx
+++ b/public/cash-flow-forecast-unze-trading.xlsx
@@ -32,9 +32,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="60" formatCode="mmm yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -67,7 +66,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,16 +398,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:M36"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="42.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -416,25 +420,40 @@
         <v/>
       </c>
       <c r="B1" s="1">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="C1" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="D1" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="E1" s="1">
-        <v>46266</v>
+        <v>46296</v>
       </c>
       <c r="F1" s="1">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="G1" s="1">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="H1" s="1">
-        <v>46357</v>
+        <v>46388</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46419</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46447</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46478</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46508</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46539</v>
       </c>
     </row>
     <row r="2">
@@ -462,9 +481,60 @@
       <c r="H2">
         <v>0</v>
       </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
         <v/>
       </c>
     </row>
@@ -472,6 +542,42 @@
       <c r="A4" t="str">
         <v>CASH INFLOW</v>
       </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -498,6 +604,21 @@
       <c r="H5">
         <v>0</v>
       </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -524,6 +645,21 @@
       <c r="H6">
         <v>0</v>
       </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -550,6 +686,21 @@
       <c r="H7">
         <v>0</v>
       </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -576,6 +727,21 @@
       <c r="H8">
         <v>0</v>
       </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -602,105 +768,230 @@
       <c r="H9">
         <v>0</v>
       </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>TOTAL INFLOW</v>
+        <v>Bank Financing</v>
       </c>
       <c r="B10">
-        <f>SUM(B5:B9)</f>
         <v>0</v>
       </c>
       <c r="C10">
-        <f>SUM(C5:C9)</f>
         <v>0</v>
       </c>
       <c r="D10">
-        <f>SUM(D5:D9)</f>
         <v>0</v>
       </c>
       <c r="E10">
-        <f>SUM(E5:E9)</f>
         <v>0</v>
       </c>
       <c r="F10">
-        <f>SUM(F5:F9)</f>
         <v>0</v>
       </c>
       <c r="G10">
-        <f>SUM(G5:G9)</f>
         <v>0</v>
       </c>
       <c r="H10">
-        <f>SUM(H5:H9)</f>
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
         <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>TOTAL INFLOW</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CASH OUTFLOW</v>
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Salaries</v>
-      </c>
-      <c r="B13">
-        <v>0</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
+        <v>CASH OUTFLOW</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Admin Expenses</v>
-      </c>
-      <c r="B14">
-        <v>0</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
-        <v>0</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
+        <v>Pole Project</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Welfare</v>
+        <v>Vendor Payments</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -721,12 +1012,27 @@
         <v>0</v>
       </c>
       <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
         <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Less: Depreciation (non-cash)</v>
+        <v>Salaries and Wages</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -747,110 +1053,185 @@
         <v>0</v>
       </c>
       <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>TOTAL OUTFLOW</v>
+        <v>Rent, retainership, Sales Tax, Utilities</v>
       </c>
       <c r="B17">
-        <f>SUM(B13:B16)</f>
         <v>0</v>
       </c>
       <c r="C17">
-        <f>SUM(C13:C16)</f>
         <v>0</v>
       </c>
       <c r="D17">
-        <f>SUM(D13:D16)</f>
         <v>0</v>
       </c>
       <c r="E17">
-        <f>SUM(E13:E16)</f>
         <v>0</v>
       </c>
       <c r="F17">
-        <f>SUM(F13:F16)</f>
         <v>0</v>
       </c>
       <c r="G17">
-        <f>SUM(G13:G16)</f>
         <v>0</v>
       </c>
       <c r="H17">
-        <f>SUM(H13:H16)</f>
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
         <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v/>
+        <v>Misc (Imprest etc)</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>NET CASH FLOW</v>
+        <v>Welfare</v>
       </c>
       <c r="B19">
-        <f>B10-B17</f>
         <v>0</v>
       </c>
       <c r="C19">
-        <f>C10-C17</f>
         <v>0</v>
       </c>
       <c r="D19">
-        <f>D10-D17</f>
         <v>0</v>
       </c>
       <c r="E19">
-        <f>E10-E17</f>
         <v>0</v>
       </c>
       <c r="F19">
-        <f>F10-F17</f>
         <v>0</v>
       </c>
       <c r="G19">
-        <f>G10-G17</f>
         <v>0</v>
       </c>
       <c r="H19">
-        <f>H10-H17</f>
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CLOSING BALANCE</v>
+        <v>Director Expense</v>
       </c>
       <c r="B20">
-        <f>B2+B19</f>
         <v>0</v>
       </c>
       <c r="C20">
-        <f>C2+C19</f>
         <v>0</v>
       </c>
       <c r="D20">
-        <f>D2+D19</f>
         <v>0</v>
       </c>
       <c r="E20">
-        <f>E2+E19</f>
         <v>0</v>
       </c>
       <c r="F20">
-        <f>F2+F19</f>
         <v>0</v>
       </c>
       <c r="G20">
-        <f>G2+G19</f>
         <v>0</v>
       </c>
       <c r="H20">
-        <f>H2+H19</f>
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20">
         <v>0</v>
       </c>
     </row>
@@ -858,15 +1239,661 @@
       <c r="A21" t="str">
         <v/>
       </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Note: Each month closing should equal next month opening. Depreciation is included as outflow but represents non-cash.</v>
+        <v>Meter Project</v>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v/>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Vendor Payments</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Salaries and Wages</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Rent, retainership, Sales Tax, Utilities</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Misc (Imprest etc)</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Welfare</v>
+      </c>
+      <c r="B27">
+        <v>0</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Warranty Claims 2%</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v/>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Bank Financing  (Payment)</v>
+      </c>
+      <c r="B30">
+        <v>0</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TOTAL OUTFLOW</v>
+      </c>
+      <c r="B31">
+        <v>0</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+      <c r="L31">
+        <v>0</v>
+      </c>
+      <c r="M31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v/>
+      </c>
+      <c r="B32" t="str">
+        <v/>
+      </c>
+      <c r="C32" t="str">
+        <v/>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
+        <v/>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>NET CASH FLOW</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
+      <c r="L33">
+        <v>0</v>
+      </c>
+      <c r="M33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>CLOSING BALANCE</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <v>0</v>
+      </c>
+      <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="M34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Note: Each month closing should equal next month opening. Pole Project and Meter Project section headings group the expense lines below them.</v>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>